<commit_message>
Update schedule to 4-block time layout and add CityPASS reservation summary
</commit_message>
<xml_diff>
--- a/ReadytoTrip.xlsx
+++ b/ReadytoTrip.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="12510" windowHeight="11060" tabRatio="500"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="25350" windowHeight="11100" tabRatio="500"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Sheet1" sheetId="1" r:id="rId4"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <x:si>
     <x:t>주아성</x:t>
   </x:si>
@@ -61,6 +61,9 @@
   </x:si>
   <x:si>
     <x:t>주이솔</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KB손해보험</x:t>
   </x:si>
   <x:si>
     <x:t>3339 Cooper Point Road Northwest, Olympia, WA 98502, United State</x:t>
@@ -155,7 +158,7 @@
       <x:patternFill patternType="gray125"/>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border>
       <x:left>
         <x:color rgb="ff000000"/>
@@ -170,42 +173,62 @@
         <x:color rgb="ff000000"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color auto="1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color auto="1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color auto="1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color auto="1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="42" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
-        <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" hs:applyExtension="1">
+        <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" hs:applyExtension="1">
           <x:alignment horizontal="center" vertical="center"/>
           <hs:parashape hs:lineSpacingType="betweenLines" hs:lineSpacing="75" hs:breakNonLatinWord="breakWord" hs:breakLatinWord="keepWord" hs:condense="0" hs:textAlignment="baseLine"/>
         </x:xf>
       </mc:Choice>
       <mc:Fallback>
-        <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+        <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
           <x:alignment horizontal="center" vertical="center"/>
         </x:xf>
       </mc:Fallback>
     </mc:AlternateContent>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="42" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -539,111 +562,115 @@
     <x:col min="5" max="8" width="16.33984375" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="2" spans="4:8">
+    <x:row r="2" spans="2:8">
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="2"/>
       <x:c r="D2" s="3" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
     </x:row>
-    <x:row r="3" spans="4:8">
+    <x:row r="3" spans="2:8">
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
       <x:c r="D3" s="3"/>
-      <x:c r="E3" t="s">
+      <x:c r="E3" s="5" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F3" t="s">
+      <x:c r="F3" s="5" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G3" t="s">
+      <x:c r="G3" s="5" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H3" t="s">
+      <x:c r="H3" s="5" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="2:8">
       <x:c r="B4" s="2" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D4" s="1">
+      <x:c r="D4" s="6">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H4" t="s">
-        <x:v>17</x:v>
+      <x:c r="E4" s="5" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="s">
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="2:8">
       <x:c r="B5" s="2"/>
-      <x:c r="C5" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="D5" s="1">
+      <x:c r="C5" s="5" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D5" s="6">
         <x:f>SUM(E5:H5)</x:f>
         <x:v>756000</x:v>
       </x:c>
-      <x:c r="E5" s="1">
+      <x:c r="E5" s="6">
         <x:v>189000</x:v>
       </x:c>
-      <x:c r="F5" s="1">
+      <x:c r="F5" s="6">
         <x:v>189000</x:v>
       </x:c>
-      <x:c r="G5" s="1">
+      <x:c r="G5" s="6">
         <x:v>189000</x:v>
       </x:c>
-      <x:c r="H5" s="1">
+      <x:c r="H5" s="6">
         <x:v>189000</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="2:8">
       <x:c r="B6" s="2"/>
-      <x:c r="C6" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="D6" s="1">
+      <x:c r="C6" s="5" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D6" s="6">
         <x:f>SUM(E6:H6)</x:f>
         <x:v>492700</x:v>
       </x:c>
-      <x:c r="E6" s="1">
+      <x:c r="E6" s="6">
         <x:v>126600</x:v>
       </x:c>
-      <x:c r="F6" s="1">
+      <x:c r="F6" s="6">
         <x:v>119600</x:v>
       </x:c>
-      <x:c r="G6" s="1">
+      <x:c r="G6" s="6">
         <x:v>126600</x:v>
       </x:c>
-      <x:c r="H6" s="1">
+      <x:c r="H6" s="6">
         <x:v>119900</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="2:8" ht="33.5" customHeight="1">
       <x:c r="B7" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D7" s="1">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D7" s="6">
         <x:v>928592</x:v>
       </x:c>
-      <x:c r="E7" s="5" t="s">
-        <x:v>9</x:v>
+      <x:c r="E7" s="8" t="s">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F7" s="2"/>
       <x:c r="G7" s="2"/>
@@ -651,14 +678,14 @@
     </x:row>
     <x:row r="8" spans="2:8" ht="32" customHeight="1">
       <x:c r="B8" s="2"/>
-      <x:c r="C8" s="6" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D8" s="1">
+      <x:c r="C8" s="7" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D8" s="6">
         <x:v>1929368</x:v>
       </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>23</x:v>
+      <x:c r="E8" s="8" t="s">
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F8" s="2"/>
       <x:c r="G8" s="2"/>
@@ -666,16 +693,16 @@
     </x:row>
     <x:row r="9" spans="2:8" ht="39.5" customHeight="1">
       <x:c r="B9" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D9" s="1">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D9" s="6">
         <x:v>277300</x:v>
       </x:c>
-      <x:c r="E9" s="5" t="s">
-        <x:v>21</x:v>
+      <x:c r="E9" s="8" t="s">
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F9" s="2"/>
       <x:c r="G9" s="2"/>
@@ -683,37 +710,52 @@
     </x:row>
     <x:row r="10" spans="2:8">
       <x:c r="B10" s="2"/>
-      <x:c r="C10" t="s">
+      <x:c r="C10" s="5" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D10" s="1">
+      <x:c r="D10" s="6">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E10" s="5" t="s">
+      <x:c r="E10" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="2"/>
       <x:c r="H10" s="2"/>
     </x:row>
-    <x:row r="11" spans="2:2">
-      <x:c r="B11" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="2:4">
-      <x:c r="B12" t="s">
+    <x:row r="11" spans="2:8">
+      <x:c r="B11" s="5" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D11" s="6">
+        <x:v>36690</x:v>
+      </x:c>
+      <x:c r="E11" s="5"/>
+      <x:c r="F11" s="5"/>
+      <x:c r="G11" s="5"/>
+      <x:c r="H11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="2:8">
+      <x:c r="B12" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C12" t="s">
+      <x:c r="C12" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D12" s="1">
+      <x:c r="D12" s="6">
         <x:v>602562</x:v>
       </x:c>
+      <x:c r="E12" s="5"/>
+      <x:c r="F12" s="5"/>
+      <x:c r="G12" s="5"/>
+      <x:c r="H12" s="5"/>
     </x:row>
   </x:sheetData>
-  <x:mergeCells count="9">
+  <x:mergeCells count="10">
+    <x:mergeCell ref="B2:C3"/>
     <x:mergeCell ref="D2:D3"/>
     <x:mergeCell ref="E2:H2"/>
     <x:mergeCell ref="B4:B6"/>

</xml_diff>